<commit_message>
update on the api routes as used in the project
</commit_message>
<xml_diff>
--- a/documentation/MLOps_UseCase_1_API_Design .xlsx
+++ b/documentation/MLOps_UseCase_1_API_Design .xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CONESTOGA\AI and ML\SEMESTER2\projects in ML\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CONESTOGA\AI and ML\SEMESTER2\projects in ML\april\NURTURE_JOY\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EA3F57F-123D-44C0-A6B3-059A9653A66C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E19E4B04-4FF4-4640-AC5B-04DB71047781}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="18" activeTab="25" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ALL_APIs" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,23 @@
     <sheet name="user_by_id-GET" sheetId="2" r:id="rId7"/>
     <sheet name="admin-delete" sheetId="5" r:id="rId8"/>
     <sheet name="update_user-PUT" sheetId="6" r:id="rId9"/>
+    <sheet name="CHAT_SERVICES &gt;" sheetId="11" r:id="rId10"/>
+    <sheet name="session_start" sheetId="13" r:id="rId11"/>
+    <sheet name="chat_message" sheetId="14" r:id="rId12"/>
+    <sheet name="chat_history" sheetId="12" r:id="rId13"/>
+    <sheet name="intent" sheetId="15" r:id="rId14"/>
+    <sheet name="session_end" sheetId="16" r:id="rId15"/>
+    <sheet name="get_user_sessions" sheetId="17" r:id="rId16"/>
+    <sheet name="delete_session" sheetId="18" r:id="rId17"/>
+    <sheet name="JOURNAL_SERVICES&gt;" sheetId="19" r:id="rId18"/>
+    <sheet name="journal_prompt" sheetId="20" r:id="rId19"/>
+    <sheet name="add_journal" sheetId="21" r:id="rId20"/>
+    <sheet name="get_journals" sheetId="22" r:id="rId21"/>
+    <sheet name="MOOD_SERVICES" sheetId="23" r:id="rId22"/>
+    <sheet name="user_mood" sheetId="24" r:id="rId23"/>
+    <sheet name="get_moods" sheetId="25" r:id="rId24"/>
+    <sheet name="mood_summary" sheetId="26" r:id="rId25"/>
+    <sheet name="Sheet17" sheetId="27" r:id="rId26"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="188">
   <si>
     <t>GET</t>
   </si>
@@ -472,6 +489,436 @@
   </si>
   <si>
     <t>Option</t>
+  </si>
+  <si>
+    <t>register a new iser session in the database</t>
+  </si>
+  <si>
+    <t>User's message (Required)</t>
+  </si>
+  <si>
+    <t>http://localhost/api/chat/session/start</t>
+  </si>
+  <si>
+    <t>Create a new chat session and send initial greeting</t>
+  </si>
+  <si>
+    <t>Bearer token (Required)</t>
+  </si>
+  <si>
+    <t>{
+  "session_id": "string",
+  "message": {
+    "id": "string",
+    "session_id": "string",
+    "role": "assistant",
+    "type": "greeting",
+    "text": "string",
+    "link": "string/null",
+    "quick_replies": [
+      { "id": "string", "label": "string" }
+    ]
+  }
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> http://localhost/api/chat/session/{session_id}/message</t>
+  </si>
+  <si>
+    <t>Send user message and receive chatbot response</t>
+  </si>
+  <si>
+    <t>session_id</t>
+  </si>
+  <si>
+    <t>Chat session ID (Path param)</t>
+  </si>
+  <si>
+    <t>text</t>
+  </si>
+  <si>
+    <t>{
+  "message": {
+    "id": "string",
+    "session_id": "string",
+    "role": "assistant",
+    "type": "chat | safety | closing",
+    "text": "string",
+    "link": "string/null",
+    "quick_replies": [
+      { "id": "string", "label": "string" }
+    ]
+  }
+}</t>
+  </si>
+  <si>
+    <t>Missing text / Session ended</t>
+  </si>
+  <si>
+    <t>{
+  "error": "Missing text/ Session ended"
+}</t>
+  </si>
+  <si>
+    <t>{
+  "error": "Invalid session"
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> http://localhost/api/chat/session/{session_id}/history</t>
+  </si>
+  <si>
+    <t>Chat session ID</t>
+  </si>
+  <si>
+    <t>{
+  "session_id": "string",
+  "turns": 5,
+  "messages": [
+    {
+      "id": "string",
+      "role": "user/assistant",
+      "type": "chat/greeting",
+      "text": "string",
+      "timestamp": "datetime"
+    }
+  ]
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> http://localhost/api/chat/session/{session_id}/intent</t>
+  </si>
+  <si>
+    <t>Handle quick reply actions (breathing, journaling, etc.)</t>
+  </si>
+  <si>
+    <t>intent</t>
+  </si>
+  <si>
+    <t>Intent ID (required)</t>
+  </si>
+  <si>
+    <t>{
+  "message": {
+    "id": "string",
+    "role": "assistant",
+    "type": "resource",
+    "text": "string",
+    "link": "string",
+    "quick_replies": [
+      { "id": "string", "label": "string" }
+    ]
+  }
+}</t>
+  </si>
+  <si>
+    <t>Missing Intent</t>
+  </si>
+  <si>
+    <t>http://localhost/api/chat/session/{session_id}/sessionend</t>
+  </si>
+  <si>
+    <t>End chat session manually</t>
+  </si>
+  <si>
+    <t>{
+  "status": "ended",
+  "session_id": "string",
+  "ended_at": "datetime"
+}</t>
+  </si>
+  <si>
+    <t>http://localhost/api/chat/sessions</t>
+  </si>
+  <si>
+    <t>Retrieve all sessions for a user</t>
+  </si>
+  <si>
+    <t>{
+  "sessions": [
+    {
+      "id": "string",
+      "created_at": "datetime",
+      "ended": true
+    }
+  ]
+}</t>
+  </si>
+  <si>
+    <t>http://localhost/api/chat/session/{session_id}</t>
+  </si>
+  <si>
+    <t>Delete a chat session and all messages</t>
+  </si>
+  <si>
+    <t>{
+  "message": "Session deleted successfully"
+}</t>
+  </si>
+  <si>
+    <t>session_ID</t>
+  </si>
+  <si>
+    <t>Not Found</t>
+  </si>
+  <si>
+    <t>{
+  "message": "Session not found"
+}</t>
+  </si>
+  <si>
+    <t>http://localhost/api/journal/prompt</t>
+  </si>
+  <si>
+    <t>Get a random journaling prompt</t>
+  </si>
+  <si>
+    <t>{
+  "prompt": "What are you grateful for today?"
+}</t>
+  </si>
+  <si>
+    <t>{
+  "prompt": "string"
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> http://localhost//api/journal</t>
+  </si>
+  <si>
+    <t>Save new journal entry</t>
+  </si>
+  <si>
+    <t>Authorization</t>
+  </si>
+  <si>
+    <t>prompt</t>
+  </si>
+  <si>
+    <t>Journal prompt (Optional)</t>
+  </si>
+  <si>
+    <t>content</t>
+  </si>
+  <si>
+    <t>journal text content (required</t>
+  </si>
+  <si>
+    <t>{
+  "message": "string",
+  "entry": {
+    "id": "integer",
+    "user_id": "integer",
+    "prompt": "string",
+    "content": "string",
+    "created_at": "datetime"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "message": "Journal saved successfully",
+  "entry": {
+    "id": 5,
+    "user_id": 2,
+    "prompt": "What are you grateful for today?",
+    "content": "I am grateful for my progress in school and my health.",
+    "created_at": "2026-04-06T14:20:00"
+  }
+}</t>
+  </si>
+  <si>
+    <t>Missing Required field</t>
+  </si>
+  <si>
+    <t>{
+  "error": "Journal conent required"
+}</t>
+  </si>
+  <si>
+    <t>Retrieve all journal entries for a user</t>
+  </si>
+  <si>
+    <t>http://localhost/api/journal</t>
+  </si>
+  <si>
+    <t>Bearer token (required)</t>
+  </si>
+  <si>
+    <t>{
+  "entries": [
+    {
+      "id": "integer",
+      "user_id": "integer",
+      "prompt": "string",
+      "content": "string",
+      "created_at": "datetime"
+    }
+  ]
+}</t>
+  </si>
+  <si>
+    <t>{
+  "entries": [
+    {
+      "id": 6,
+      "user_id": 2,
+      "prompt": "What is one small win you had today?",
+      "content": "I completed my assignment on time.",
+      "created_at": "2026-04-06T13:00:00"
+    },
+    {
+      "id": 5,
+      "user_id": 2,
+      "prompt": "What are you grateful for today?",
+      "content": "I am grateful for my progress in school.",
+      "created_at": "2026-04-05T18:00:00"
+    }
+  ]
+}</t>
+  </si>
+  <si>
+    <t>{
+  "error": "string"
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> http://localhost/api/mood/track</t>
+  </si>
+  <si>
+    <t>Track/Log a user's mood</t>
+  </si>
+  <si>
+    <t>mood</t>
+  </si>
+  <si>
+    <t>Mood type (required)</t>
+  </si>
+  <si>
+    <t>intensity</t>
+  </si>
+  <si>
+    <t>Mood intensity (optional)</t>
+  </si>
+  <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>Additional note(optional)</t>
+  </si>
+  <si>
+    <t>{
+  "message": "string",
+  "mood": {
+    "id": "integer",
+    "user_id": "integer",
+    "mood": "string",
+    "intensity": "integer",
+    "note": "string",
+    "created_at": "datetime"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "message": "Mood logged successfully",
+  "mood": {
+    "id": 12,
+    "user_id": 3,
+    "mood": "happy",
+    "intensity": 8,
+    "note": "Had a really productive day!",
+    "created_at": "2026-04-06T15:00:00"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "error": "Mood required"
+}</t>
+  </si>
+  <si>
+    <t>Retrieve all mood logs for a user</t>
+  </si>
+  <si>
+    <t>http://localhost/api/mood/history</t>
+  </si>
+  <si>
+    <t>{
+  "moods": [
+    {
+      "id": "integer",
+      "user_id": "integer",
+      "mood": "string",
+      "intensity": "integer",
+      "note": "string",
+      "created_at": "datetime"
+    }
+  ]
+}</t>
+  </si>
+  <si>
+    <t>{
+  "moods": [
+    {
+      "id": 12,
+      "user_id": 3,
+      "mood": "happy",
+      "intensity": 8,
+      "note": "Had a great day",
+      "created_at": "2026-04-06T15:00:00"
+    },
+    {
+      "id": 11,
+      "user_id": 3,
+      "mood": "anxious",
+      "intensity": 6,
+      "note": "Feeling a bit stressed",
+      "created_at": "2026-04-05T20:00:00"
+    }
+  ]
+}</t>
+  </si>
+  <si>
+    <t>Get mood frequency summary (counts per mood type)</t>
+  </si>
+  <si>
+    <t>http://localhost/api/mood/summary</t>
+  </si>
+  <si>
+    <t>{
+  "summary": {
+    "mood_type": "integer"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "moods": [{
+  "summary": {
+    "happy": 5,
+    "anxious": 3,
+    "sad": 2
+  }
+}
+    {
+      "id": 12,
+      "user_id": 3,
+      "mood": "happy",
+      "intensity": 8,
+      "note": "Had a great day",
+      "created_at": "2026-04-06T15:00:00"
+    },
+    {
+      "id": 11,
+      "user_id": 3,
+      "mood": "anxious",
+      "intensity": 6,
+      "note": "Feeling a bit stressed",
+      "created_at": "2026-04-05T20:00:00"
+    }
+  ]
+}</t>
   </si>
 </sst>
 </file>
@@ -577,7 +1024,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -606,15 +1053,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -624,10 +1062,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -637,29 +1071,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -678,6 +1091,46 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1013,7 +1466,7 @@
       <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="4" t="s">
@@ -1165,7 +1618,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -1193,6 +1646,930 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B468222A-689E-40C6-8522-003E519265ED}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF5602BE-6F7B-4394-BC5C-B444EA1ACB90}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="32.08984375" customWidth="1"/>
+    <col min="2" max="2" width="39.90625" customWidth="1"/>
+    <col min="3" max="3" width="50.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="13"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="13"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="1">
+        <v>200</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="203" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="B9" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>401</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="3"/>
+      <c r="B11" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B1" r:id="rId1" xr:uid="{156F6822-9ADE-42D7-A4D6-AEE3E3CAA24C}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C5903B-C6C2-451B-B55A-A9A2F8732B29}">
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr defaultColWidth="49.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="16384" width="49.54296875" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="26"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C4" s="15"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C5" s="15"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="26"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="6">
+        <v>201</v>
+      </c>
+      <c r="B8" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="32"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="6"/>
+      <c r="B9" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="C10" s="6"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="6">
+        <v>400</v>
+      </c>
+      <c r="B11" s="32" t="s">
+        <v>124</v>
+      </c>
+      <c r="C11" s="32"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="12"/>
+      <c r="B12" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="12"/>
+      <c r="B13" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="12">
+        <v>404</v>
+      </c>
+      <c r="B14" s="31" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="31"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="12"/>
+      <c r="B15" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A16" s="12"/>
+      <c r="B16" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B11:C11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5633F3E-9001-4F4A-8F9A-DB8ECA207D55}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultColWidth="49.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="16384" width="49.54296875" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="26"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="C4" s="15"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="23"/>
+      <c r="C5" s="23"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="26"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="6">
+        <v>201</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="32"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="6"/>
+      <c r="B8" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C9" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1417FD5-BF69-46FF-B4B6-120F8D03D2E3}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultColWidth="49.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="16384" width="49.54296875" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="26"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C4" s="15"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="23"/>
+      <c r="C5" s="23"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="26"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="6">
+        <v>201</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="32"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="6"/>
+      <c r="B8" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="174" x14ac:dyDescent="0.35">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="C9" s="6"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="6">
+        <v>400</v>
+      </c>
+      <c r="B10" s="32" t="s">
+        <v>135</v>
+      </c>
+      <c r="C10" s="32"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B10:C10"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A241D4D4-FB45-40AC-9DE4-1470856AE845}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultColWidth="25.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.90625" style="4"/>
+    <col min="2" max="2" width="42.7265625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="45.7265625" style="4" customWidth="1"/>
+    <col min="4" max="16384" width="25.90625" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="13"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="13"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="1">
+        <v>200</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="B9" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C9" s="2"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B1" r:id="rId1" xr:uid="{FAC1AA07-F780-48C7-8454-8B4B44395758}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{513A4055-92DC-4D0C-A5DD-336233D02C69}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="27.26953125" customWidth="1"/>
+    <col min="2" max="2" width="40.08984375" customWidth="1"/>
+    <col min="3" max="3" width="45.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="13"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="13"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="1">
+        <v>200</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="B9" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C9" s="2"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B1" r:id="rId1" xr:uid="{AD5E810D-E23A-43B4-A0A6-90D1BDCA56B7}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{804E37EC-6B1D-419D-ABF9-8DCB1D915F0E}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="23.90625" customWidth="1"/>
+    <col min="2" max="2" width="46.1796875" customWidth="1"/>
+    <col min="3" max="3" width="36.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="25"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="1"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="25"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="1">
+        <v>200</v>
+      </c>
+      <c r="B8" s="33" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="33"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="1"/>
+      <c r="B9" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="58" x14ac:dyDescent="0.35">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="1">
+        <v>404</v>
+      </c>
+      <c r="B11" s="33" t="s">
+        <v>146</v>
+      </c>
+      <c r="C11" s="33"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="1"/>
+      <c r="B12" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C14" s="34"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B1" r:id="rId1" xr:uid="{1A983EC4-4112-4CD7-99CB-B6B4F4253D9C}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A50FA37F-6C89-43E3-9E42-D9443EC1D877}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E55E8C36-BF2D-4876-B099-44777A5862A7}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="27.26953125" customWidth="1"/>
+    <col min="2" max="2" width="40.08984375" customWidth="1"/>
+    <col min="3" max="3" width="45.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="C1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="13"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="13"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="1">
+        <v>200</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="B9" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B1" r:id="rId1" xr:uid="{A66A3F70-BD9D-404F-8AE0-F4C970305EF3}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1218,20 +2595,20 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="11"/>
+      <c r="C3" s="30"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
@@ -1279,29 +2656,29 @@
       <c r="C8" s="7"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
+      <c r="B9" s="29"/>
+      <c r="C9" s="29"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="11"/>
+      <c r="C10" s="30"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="9">
         <v>201</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="12"/>
+      <c r="C11" s="28"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="9"/>
@@ -1325,53 +2702,53 @@
       <c r="A14" s="9">
         <v>400</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="C14" s="12"/>
+      <c r="C14" s="28"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="13"/>
-      <c r="B15" s="14" t="s">
+      <c r="A15" s="10"/>
+      <c r="B15" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="11" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="13"/>
-      <c r="B16" s="15" t="s">
+      <c r="A16" s="10"/>
+      <c r="B16" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="12" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="13">
+      <c r="A17" s="10">
         <v>409</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="C17" s="16"/>
+      <c r="C17" s="27"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14" t="s">
+      <c r="A18" s="10"/>
+      <c r="B18" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="11" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="13"/>
-      <c r="B19" s="15" t="s">
+      <c r="A19" s="10"/>
+      <c r="B19" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="12" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1389,18 +2766,765 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E22D6686-9F6F-4BFB-A5FA-DC6EBC04B15D}">
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.54296875" customWidth="1"/>
+    <col min="2" max="2" width="47.81640625" customWidth="1"/>
+    <col min="3" max="3" width="47.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="26"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="35" t="s">
+        <v>154</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C4" s="15"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="35" t="s">
+        <v>155</v>
+      </c>
+      <c r="B5" t="s">
+        <v>156</v>
+      </c>
+      <c r="C5" s="15"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="35" t="s">
+        <v>157</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="C6" s="15"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="26"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="6">
+        <v>201</v>
+      </c>
+      <c r="B9" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="32"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="6"/>
+      <c r="B10" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="6">
+        <v>400</v>
+      </c>
+      <c r="B12" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="C12" s="32"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="12"/>
+      <c r="B13" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="12"/>
+      <c r="B14" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="12">
+        <v>401</v>
+      </c>
+      <c r="B15" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="C15" s="31"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="12"/>
+      <c r="B16" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A17" s="12"/>
+      <c r="B17" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B12:C12"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17FBE490-2E60-4130-9272-3D31894F2540}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="27.26953125" customWidth="1"/>
+    <col min="2" max="2" width="40.08984375" customWidth="1"/>
+    <col min="3" max="3" width="45.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="C1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="13"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="13"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="1">
+        <v>200</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="290" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="B9" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="1">
+        <v>401</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10" s="1"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="2"/>
+      <c r="B11" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="2"/>
+      <c r="B12" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B1" r:id="rId1" xr:uid="{AEC92666-0432-4E52-9A90-AD9990188F8E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB0704A9-081B-4023-8271-C34FB1433095}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADC1FFAE-AA7F-4522-A7A0-13509738526D}">
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="27.453125" customWidth="1"/>
+    <col min="2" max="2" width="33.453125" customWidth="1"/>
+    <col min="3" max="3" width="31.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="26"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="35" t="s">
+        <v>154</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C4" s="15"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C5" s="15"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="35" t="s">
+        <v>173</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="C6" s="15"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="36" t="s">
+        <v>175</v>
+      </c>
+      <c r="B7" t="s">
+        <v>176</v>
+      </c>
+      <c r="C7" s="15"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="26"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="6">
+        <v>201</v>
+      </c>
+      <c r="B10" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="32"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="6"/>
+      <c r="B11" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="203" x14ac:dyDescent="0.35">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="6">
+        <v>400</v>
+      </c>
+      <c r="B13" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="C13" s="32"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="12"/>
+      <c r="B14" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="12"/>
+      <c r="B15" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="12">
+        <v>401</v>
+      </c>
+      <c r="B16" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16" s="31"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="12"/>
+      <c r="B17" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="12"/>
+      <c r="B18" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B13:C13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCDA9110-5EEE-4CAD-94A4-147CCD457261}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="31.90625" customWidth="1"/>
+    <col min="2" max="2" width="33.54296875" customWidth="1"/>
+    <col min="3" max="3" width="37.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="13"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="13"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="1">
+        <v>200</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="290" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="B9" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="1">
+        <v>401</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10" s="1"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="2"/>
+      <c r="B11" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="2"/>
+      <c r="B12" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B1" r:id="rId1" xr:uid="{D20F1378-82D7-4047-AAA7-B47EC2748AD4}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A471E54-3D4F-4B6D-9A8E-D958E69183C5}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="31.90625" customWidth="1"/>
+    <col min="2" max="2" width="33.54296875" customWidth="1"/>
+    <col min="3" max="3" width="37.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="13"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="13"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="1">
+        <v>200</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="377" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="B9" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="1">
+        <v>401</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10" s="1"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="2"/>
+      <c r="B11" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="2"/>
+      <c r="B12" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B1" r:id="rId1" xr:uid="{703929F6-E3B9-4479-AB92-45F36B6DAF83}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6C12D31-9003-400E-8545-FB3C47416FFD}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC3458BC-11C9-484B-B4E2-3D919EC7D4D2}">
   <dimension ref="A1:C19"/>
   <sheetFormatPr defaultColWidth="36.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="36.26953125" style="17"/>
-    <col min="3" max="3" width="46.81640625" style="17" customWidth="1"/>
-    <col min="4" max="16384" width="36.26953125" style="17"/>
+    <col min="3" max="3" width="46.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="15" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="8" t="s">
@@ -1411,20 +3535,20 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="22"/>
+      <c r="C3" s="26"/>
     </row>
     <row r="4" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
@@ -1433,7 +3557,7 @@
       <c r="B4" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C4" s="20"/>
+      <c r="C4" s="15"/>
     </row>
     <row r="5" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
@@ -1442,39 +3566,39 @@
       <c r="B5" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C5" s="20"/>
+      <c r="C5" s="15"/>
     </row>
     <row r="6" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="22"/>
+      <c r="C7" s="26"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="6">
         <v>200</v>
       </c>
-      <c r="B8" s="23" t="s">
+      <c r="B8" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="23"/>
+      <c r="C8" s="32"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="6"/>
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="15" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1491,80 +3615,80 @@
       <c r="A11" s="6">
         <v>400</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="C11" s="23"/>
+      <c r="C11" s="32"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="15"/>
-      <c r="B12" s="24" t="s">
+      <c r="A12" s="12"/>
+      <c r="B12" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="24" t="s">
+      <c r="C12" s="16" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="15"/>
-      <c r="B13" s="15" t="s">
+      <c r="A13" s="12"/>
+      <c r="B13" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="12" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="15">
+      <c r="A14" s="12">
         <v>401</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="C14" s="25"/>
+      <c r="C14" s="31"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="15"/>
-      <c r="B15" s="24" t="s">
+      <c r="A15" s="12"/>
+      <c r="B15" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="24" t="s">
+      <c r="C15" s="16" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="15"/>
-      <c r="B16" s="15" t="s">
+      <c r="A16" s="12"/>
+      <c r="B16" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="12" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="15">
+      <c r="A17" s="12">
         <v>404</v>
       </c>
-      <c r="B17" s="25" t="s">
+      <c r="B17" s="31" t="s">
         <v>78</v>
       </c>
-      <c r="C17" s="25"/>
+      <c r="C17" s="31"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" s="15"/>
-      <c r="B18" s="24" t="s">
+      <c r="A18" s="12"/>
+      <c r="B18" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="24" t="s">
+      <c r="C18" s="16" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="15"/>
-      <c r="B19" s="15" t="s">
+      <c r="A19" s="12"/>
+      <c r="B19" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="12" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1592,7 +3716,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
@@ -1603,20 +3727,20 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="27"/>
+      <c r="C3" s="25"/>
     </row>
     <row r="4" spans="1:3" ht="32.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
@@ -1625,39 +3749,39 @@
       <c r="B4" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="C4" s="18"/>
+      <c r="C4" s="13"/>
     </row>
     <row r="5" spans="1:3" ht="21.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="27"/>
+      <c r="C6" s="25"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>200</v>
       </c>
-      <c r="B7" s="28" t="s">
+      <c r="B7" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="28"/>
+      <c r="C7" s="33"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="13" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1674,17 +3798,17 @@
       <c r="A10" s="1">
         <v>401</v>
       </c>
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="28"/>
+      <c r="C10" s="33"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="2"/>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="14" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1699,12 +3823,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="B10:C10"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B10:C10"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B1" r:id="rId1" xr:uid="{E28D25D5-F57A-4578-8810-0825B2EB143E}"/>
@@ -1724,7 +3848,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
@@ -1735,20 +3859,20 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="27"/>
+      <c r="C3" s="25"/>
     </row>
     <row r="4" spans="1:3" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
@@ -1757,39 +3881,39 @@
       <c r="B4" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="C4" s="18"/>
+      <c r="C4" s="13"/>
     </row>
     <row r="5" spans="1:3" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="27"/>
+      <c r="C6" s="25"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>200</v>
       </c>
-      <c r="B7" s="28" t="s">
+      <c r="B7" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="28"/>
+      <c r="C7" s="33"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="13" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1806,17 +3930,17 @@
       <c r="A10" s="1">
         <v>401</v>
       </c>
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="28"/>
+      <c r="C10" s="33"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="2"/>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="14" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1831,12 +3955,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="B10:C10"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B10:C10"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B1" r:id="rId1" xr:uid="{08648DF6-1558-4977-9597-A491557434ED}"/>
@@ -1856,7 +3980,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="13" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="5" t="s">
@@ -1867,20 +3991,20 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="27"/>
+      <c r="C3" s="25"/>
     </row>
     <row r="4" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
@@ -1889,39 +4013,39 @@
       <c r="B4" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C4" s="18"/>
+      <c r="C4" s="13"/>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="27"/>
+      <c r="C6" s="25"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>200</v>
       </c>
-      <c r="B7" s="28" t="s">
+      <c r="B7" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="28"/>
+      <c r="C7" s="33"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="13" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1938,17 +4062,17 @@
       <c r="A10" s="1">
         <v>401</v>
       </c>
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="28"/>
+      <c r="C10" s="33"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="2"/>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="14" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1963,12 +4087,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="B10:C10"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B10:C10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1985,7 +4109,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
@@ -1996,20 +4120,20 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="18"/>
+      <c r="C3" s="13"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -2021,20 +4145,20 @@
       <c r="C4" s="1"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="29"/>
-      <c r="C5" s="29"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="18"/>
+      <c r="C6" s="13"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
@@ -2047,10 +4171,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="2"/>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="14" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2074,10 +4198,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3"/>
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="30" t="s">
+      <c r="C11" s="18" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2109,7 +4233,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="13" t="s">
         <v>53</v>
       </c>
       <c r="B1" s="5" t="s">
@@ -2120,20 +4244,20 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="27"/>
+      <c r="C3" s="25"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
@@ -2154,36 +4278,36 @@
       <c r="C5" s="1"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="27"/>
+      <c r="C7" s="25"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>200</v>
       </c>
-      <c r="B8" s="28" t="s">
+      <c r="B8" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="28"/>
+      <c r="C8" s="33"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="13" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2200,17 +4324,17 @@
       <c r="A11" s="1">
         <v>401</v>
       </c>
-      <c r="B11" s="28" t="s">
+      <c r="B11" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="C11" s="28"/>
+      <c r="C11" s="33"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="13" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2227,17 +4351,17 @@
       <c r="A14" s="1">
         <v>403</v>
       </c>
-      <c r="B14" s="28" t="s">
+      <c r="B14" s="33" t="s">
         <v>96</v>
       </c>
-      <c r="C14" s="28"/>
+      <c r="C14" s="33"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="13" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2278,7 +4402,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="15" t="s">
         <v>98</v>
       </c>
       <c r="B1" s="8" t="s">
@@ -2289,20 +4413,20 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="22"/>
+      <c r="C3" s="26"/>
     </row>
     <row r="4" spans="1:3" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
@@ -2311,7 +4435,7 @@
       <c r="B4" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="20"/>
+      <c r="C4" s="15"/>
     </row>
     <row r="5" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
@@ -2320,14 +4444,14 @@
       <c r="B5" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C5" s="20"/>
+      <c r="C5" s="15"/>
     </row>
     <row r="6" spans="1:3" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
     </row>
     <row r="7" spans="1:3" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
@@ -2336,7 +4460,7 @@
       <c r="B7" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C7" s="20"/>
+      <c r="C7" s="15"/>
     </row>
     <row r="8" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
@@ -2345,7 +4469,7 @@
       <c r="B8" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="C8" s="20"/>
+      <c r="C8" s="15"/>
     </row>
     <row r="9" spans="1:3" ht="21.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
@@ -2354,7 +4478,7 @@
       <c r="B9" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="C9" s="20"/>
+      <c r="C9" s="15"/>
     </row>
     <row r="10" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
@@ -2363,7 +4487,7 @@
       <c r="B10" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="C10" s="20"/>
+      <c r="C10" s="15"/>
     </row>
     <row r="11" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
@@ -2372,43 +4496,43 @@
       <c r="B11" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="C11" s="20"/>
+      <c r="C11" s="15"/>
     </row>
     <row r="12" spans="1:3" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
     </row>
     <row r="13" spans="1:3" ht="21.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="27" t="s">
+      <c r="B13" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="27"/>
+      <c r="C13" s="25"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>200</v>
       </c>
-      <c r="B14" s="31" t="s">
+      <c r="B14" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="C14" s="32"/>
+      <c r="C14" s="20"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="14" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="145" x14ac:dyDescent="0.35">
       <c r="A16" s="2"/>
       <c r="B16" s="4" t="s">
         <v>64</v>
@@ -2421,17 +4545,17 @@
       <c r="A17" s="2">
         <v>401</v>
       </c>
-      <c r="B17" s="33" t="s">
+      <c r="B17" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="C17" s="34"/>
+      <c r="C17" s="22"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="3"/>
-      <c r="B18" s="30" t="s">
+      <c r="B18" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="30" t="s">
+      <c r="C18" s="18" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2448,17 +4572,17 @@
       <c r="A20" s="2">
         <v>403</v>
       </c>
-      <c r="B20" s="33" t="s">
+      <c r="B20" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="C20" s="34"/>
+      <c r="C20" s="22"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
-      <c r="B21" s="30" t="s">
+      <c r="B21" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="30" t="s">
+      <c r="C21" s="18" t="s">
         <v>43</v>
       </c>
     </row>

</xml_diff>